<commit_message>
finished checking all those that has been manually coded
</commit_message>
<xml_diff>
--- a/1_Data/Constable_2019_JEPHPP/Exp1/CodeBook_Constable_2019_JEPHPP_Exp1_Clean.xlsx
+++ b/1_Data/Constable_2019_JEPHPP/Exp1/CodeBook_Constable_2019_JEPHPP_Exp1_Clean.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -639,7 +639,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Stranger;Self</t>
+          <t>Individual_Self;Group-Self;Individual_Stranger;Group-Stranger</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -832,12 +832,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Accuracy of the participant's response</t>
+          <t>Accuracy of the participant's response. Coding: 1 = correct (key matches the correct key); 0 = incorrect (key within response keys but wrong); NA = no response; -2 = out-of-range key (key outside the allowed response keys); -3 = early response (before stimulus onset); -4 = late response (after response window)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1;0;3</t>
+          <t>1 (correct); 0 (incorrect); NA (no response); -2 (out-of-range key); -3 (early response); -4 (late response)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">

</xml_diff>